<commit_message>
datos: actualización automática 2026-08-19
</commit_message>
<xml_diff>
--- a/idecba/canastas.xlsx
+++ b/idecba/canastas.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14655" windowHeight="8595"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25635" windowHeight="3345"/>
   </bookViews>
   <sheets>
     <sheet name="Canasta_cons_hogar1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="63">
   <si>
     <t>Cereales y legumbres</t>
   </si>
@@ -250,20 +250,6 @@
   </si>
   <si>
     <r>
-      <t>Evolución de su valor en pesos. Hogar 1</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>a</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <rPr>
         <b/>
         <sz val="8"/>
@@ -310,7 +296,26 @@
     <t>Canastas de consumo de la CABA</t>
   </si>
   <si>
-    <t>Canastas de consumo de la Ciudad de Buenos Aires. Enero de 2013 / marzo de 2026</t>
+    <r>
+      <t>Canastas de consumo de la Ciudad de Buenos Aires. Evolución de su valor en pesos. Hogar 1</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>a</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>. Enero de 2013 / julio 2026</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2344,7 +2349,7 @@
     <xf numFmtId="0" fontId="1" fillId="56" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="57" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="46" fillId="26" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="47" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2424,6 +2429,9 @@
     </xf>
     <xf numFmtId="0" fontId="45" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="27" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="45" fillId="27" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3391,9 +3399,9 @@
     <col min="79" max="16384" width="11.42578125" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:160" ht="15" customHeight="1">
+    <row r="1" spans="1:164" ht="15" customHeight="1">
       <c r="A1" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -3418,14 +3426,12 @@
       <c r="V1" s="15"/>
       <c r="W1" s="15"/>
     </row>
-    <row r="2" spans="1:160" s="18" customFormat="1" ht="15" customHeight="1">
-      <c r="A2" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
+    <row r="2" spans="1:164" s="18" customFormat="1" ht="15" customHeight="1">
+      <c r="A2" s="36"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
       <c r="F2" s="17"/>
       <c r="G2" s="17"/>
       <c r="H2" s="17"/>
@@ -3445,7 +3451,7 @@
       <c r="V2" s="17"/>
       <c r="W2" s="17"/>
     </row>
-    <row r="3" spans="1:160" ht="15" customHeight="1">
+    <row r="3" spans="1:164" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>22</v>
       </c>
@@ -3926,8 +3932,20 @@
       <c r="FD3" s="5">
         <v>46082</v>
       </c>
+      <c r="FE3" s="5">
+        <v>46113</v>
+      </c>
+      <c r="FF3" s="5">
+        <v>46143</v>
+      </c>
+      <c r="FG3" s="5">
+        <v>46174</v>
+      </c>
+      <c r="FH3" s="5">
+        <v>46204</v>
+      </c>
     </row>
-    <row r="4" spans="1:160" ht="12.75" customHeight="1">
+    <row r="4" spans="1:164" ht="12.75" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
@@ -4408,8 +4426,20 @@
       <c r="FD4" s="7">
         <v>220795.26</v>
       </c>
+      <c r="FE4" s="7">
+        <v>226489.5</v>
+      </c>
+      <c r="FF4" s="7">
+        <v>231855.43</v>
+      </c>
+      <c r="FG4" s="7">
+        <v>235975.45</v>
+      </c>
+      <c r="FH4" s="7">
+        <v>240504.8</v>
+      </c>
     </row>
-    <row r="5" spans="1:160" ht="12.75" customHeight="1">
+    <row r="5" spans="1:164" ht="12.75" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
@@ -4890,8 +4920,20 @@
       <c r="FD5" s="7">
         <v>188581</v>
       </c>
+      <c r="FE5" s="7">
+        <v>183513.33</v>
+      </c>
+      <c r="FF5" s="7">
+        <v>200600.33</v>
+      </c>
+      <c r="FG5" s="7">
+        <v>207051.87</v>
+      </c>
+      <c r="FH5" s="7">
+        <v>226072.85</v>
+      </c>
     </row>
-    <row r="6" spans="1:160" ht="12.75" customHeight="1">
+    <row r="6" spans="1:164" ht="12.75" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
@@ -5372,10 +5414,22 @@
       <c r="FD6" s="7">
         <v>289438.77</v>
       </c>
+      <c r="FE6" s="7">
+        <v>292659.03000000003</v>
+      </c>
+      <c r="FF6" s="7">
+        <v>292428.28000000003</v>
+      </c>
+      <c r="FG6" s="7">
+        <v>294416.31</v>
+      </c>
+      <c r="FH6" s="7">
+        <v>294091.18</v>
+      </c>
     </row>
-    <row r="7" spans="1:160" ht="12.75" customHeight="1">
+    <row r="7" spans="1:164" ht="12.75" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B7" s="6">
         <v>359.65</v>
@@ -5854,8 +5908,20 @@
       <c r="FD7" s="7">
         <v>112342.2</v>
       </c>
+      <c r="FE7" s="7">
+        <v>116017.97</v>
+      </c>
+      <c r="FF7" s="7">
+        <v>121904.11</v>
+      </c>
+      <c r="FG7" s="7">
+        <v>124749.97</v>
+      </c>
+      <c r="FH7" s="7">
+        <v>128513.31</v>
+      </c>
     </row>
-    <row r="8" spans="1:160" ht="12.75" customHeight="1">
+    <row r="8" spans="1:164" ht="12.75" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>3</v>
       </c>
@@ -6336,8 +6402,20 @@
       <c r="FD8" s="7">
         <v>23027.05</v>
       </c>
+      <c r="FE8" s="7">
+        <v>23581.3</v>
+      </c>
+      <c r="FF8" s="7">
+        <v>24316.43</v>
+      </c>
+      <c r="FG8" s="7">
+        <v>24655.919999999998</v>
+      </c>
+      <c r="FH8" s="7">
+        <v>24892.34</v>
+      </c>
     </row>
-    <row r="9" spans="1:160" ht="12.75" customHeight="1">
+    <row r="9" spans="1:164" ht="12.75" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
@@ -6818,8 +6896,20 @@
       <c r="FD9" s="8">
         <v>13662.7</v>
       </c>
+      <c r="FE9" s="8">
+        <v>14130.34</v>
+      </c>
+      <c r="FF9" s="8">
+        <v>14598.9</v>
+      </c>
+      <c r="FG9" s="8">
+        <v>14874.31</v>
+      </c>
+      <c r="FH9" s="8">
+        <v>15030.22</v>
+      </c>
     </row>
-    <row r="10" spans="1:160" ht="12.75" customHeight="1">
+    <row r="10" spans="1:164" ht="12.75" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>26</v>
       </c>
@@ -7300,8 +7390,20 @@
       <c r="FD10" s="8">
         <v>20279.8</v>
       </c>
+      <c r="FE10" s="8">
+        <v>20484.939999999999</v>
+      </c>
+      <c r="FF10" s="8">
+        <v>20817.509999999998</v>
+      </c>
+      <c r="FG10" s="8">
+        <v>20985.19</v>
+      </c>
+      <c r="FH10" s="8">
+        <v>21328.84</v>
+      </c>
     </row>
-    <row r="11" spans="1:160" ht="12.75" customHeight="1">
+    <row r="11" spans="1:164" ht="12.75" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
@@ -7782,8 +7884,20 @@
       <c r="FD11" s="8">
         <v>18230.060000000001</v>
       </c>
+      <c r="FE11" s="8">
+        <v>18369.71</v>
+      </c>
+      <c r="FF11" s="8">
+        <v>18793.02</v>
+      </c>
+      <c r="FG11" s="8">
+        <v>19061.36</v>
+      </c>
+      <c r="FH11" s="8">
+        <v>18789.5</v>
+      </c>
     </row>
-    <row r="12" spans="1:160" ht="12.75" customHeight="1">
+    <row r="12" spans="1:164" ht="12.75" customHeight="1">
       <c r="A12" s="3" t="s">
         <v>23</v>
       </c>
@@ -8264,8 +8378,20 @@
       <c r="FD12" s="10">
         <v>886356.84</v>
       </c>
+      <c r="FE12" s="10">
+        <v>895246.12</v>
+      </c>
+      <c r="FF12" s="10">
+        <v>925314.02</v>
+      </c>
+      <c r="FG12" s="10">
+        <v>941770.38</v>
+      </c>
+      <c r="FH12" s="10">
+        <v>969223.04</v>
+      </c>
     </row>
-    <row r="13" spans="1:160" ht="12.75" customHeight="1">
+    <row r="13" spans="1:164" ht="12.75" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>6</v>
       </c>
@@ -8746,8 +8872,20 @@
       <c r="FD13" s="7">
         <v>0</v>
       </c>
+      <c r="FE13" s="7">
+        <v>0</v>
+      </c>
+      <c r="FF13" s="7">
+        <v>0</v>
+      </c>
+      <c r="FG13" s="7">
+        <v>0</v>
+      </c>
+      <c r="FH13" s="7">
+        <v>0</v>
+      </c>
     </row>
-    <row r="14" spans="1:160" ht="12.75" customHeight="1">
+    <row r="14" spans="1:164" ht="12.75" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>7</v>
       </c>
@@ -9228,8 +9366,20 @@
       <c r="FD14" s="7">
         <v>138311.13</v>
       </c>
+      <c r="FE14" s="7">
+        <v>142215.12</v>
+      </c>
+      <c r="FF14" s="7">
+        <v>145267.41</v>
+      </c>
+      <c r="FG14" s="7">
+        <v>147580.22</v>
+      </c>
+      <c r="FH14" s="7">
+        <v>151417.81</v>
+      </c>
     </row>
-    <row r="15" spans="1:160" ht="12.75" customHeight="1">
+    <row r="15" spans="1:164" ht="12.75" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>9</v>
       </c>
@@ -9710,8 +9860,20 @@
       <c r="FD15" s="7">
         <v>19545.77</v>
       </c>
+      <c r="FE15" s="7">
+        <v>18774.189999999999</v>
+      </c>
+      <c r="FF15" s="7">
+        <v>18994.060000000001</v>
+      </c>
+      <c r="FG15" s="7">
+        <v>19206.14</v>
+      </c>
+      <c r="FH15" s="7">
+        <v>19435.02</v>
+      </c>
     </row>
-    <row r="16" spans="1:160" ht="12.75" customHeight="1">
+    <row r="16" spans="1:164" ht="12.75" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>8</v>
       </c>
@@ -10192,8 +10354,20 @@
       <c r="FD16" s="7">
         <v>25681.93</v>
       </c>
+      <c r="FE16" s="7">
+        <v>25999.02</v>
+      </c>
+      <c r="FF16" s="7">
+        <v>26358.35</v>
+      </c>
+      <c r="FG16" s="7">
+        <v>26823.54</v>
+      </c>
+      <c r="FH16" s="7">
+        <v>28413.98</v>
+      </c>
     </row>
-    <row r="17" spans="1:160" ht="12.75" customHeight="1">
+    <row r="17" spans="1:164" ht="12.75" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>10</v>
       </c>
@@ -10674,8 +10848,20 @@
       <c r="FD17" s="7">
         <v>40957.71</v>
       </c>
+      <c r="FE17" s="7">
+        <v>42596.01</v>
+      </c>
+      <c r="FF17" s="7">
+        <v>43873.89</v>
+      </c>
+      <c r="FG17" s="7">
+        <v>45190.11</v>
+      </c>
+      <c r="FH17" s="7">
+        <v>46838.53</v>
+      </c>
     </row>
-    <row r="18" spans="1:160" ht="12.75" customHeight="1">
+    <row r="18" spans="1:164" ht="12.75" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -11156,8 +11342,20 @@
       <c r="FD18" s="7">
         <v>51834.57</v>
       </c>
+      <c r="FE18" s="7">
+        <v>53934.49</v>
+      </c>
+      <c r="FF18" s="7">
+        <v>56068.37</v>
+      </c>
+      <c r="FG18" s="7">
+        <v>59062.91</v>
+      </c>
+      <c r="FH18" s="7">
+        <v>61810.09</v>
+      </c>
     </row>
-    <row r="19" spans="1:160" ht="12.75" customHeight="1">
+    <row r="19" spans="1:164" ht="12.75" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>11</v>
       </c>
@@ -11638,8 +11836,20 @@
       <c r="FD19" s="7">
         <v>83542.27</v>
       </c>
+      <c r="FE19" s="7">
+        <v>86486.26</v>
+      </c>
+      <c r="FF19" s="7">
+        <v>89567.29</v>
+      </c>
+      <c r="FG19" s="7">
+        <v>90045.69</v>
+      </c>
+      <c r="FH19" s="7">
+        <v>90970.64</v>
+      </c>
     </row>
-    <row r="20" spans="1:160" ht="12.75" customHeight="1">
+    <row r="20" spans="1:164" ht="12.75" customHeight="1">
       <c r="A20" s="3" t="s">
         <v>24</v>
       </c>
@@ -12120,8 +12330,20 @@
       <c r="FD20" s="10">
         <v>1246230.22</v>
       </c>
+      <c r="FE20" s="10">
+        <v>1265251.21</v>
+      </c>
+      <c r="FF20" s="10">
+        <v>1305443.3899999999</v>
+      </c>
+      <c r="FG20" s="10">
+        <v>1329678.98</v>
+      </c>
+      <c r="FH20" s="10">
+        <v>1368109.1</v>
+      </c>
     </row>
-    <row r="21" spans="1:160" ht="12.75" customHeight="1">
+    <row r="21" spans="1:164" ht="12.75" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>12</v>
       </c>
@@ -12602,8 +12824,20 @@
       <c r="FD21" s="7">
         <v>94719.13</v>
       </c>
+      <c r="FE21" s="7">
+        <v>95142.66</v>
+      </c>
+      <c r="FF21" s="7">
+        <v>98874.64</v>
+      </c>
+      <c r="FG21" s="7">
+        <v>99220.53</v>
+      </c>
+      <c r="FH21" s="7">
+        <v>103862.72</v>
+      </c>
     </row>
-    <row r="22" spans="1:160" ht="12.75" customHeight="1">
+    <row r="22" spans="1:164" ht="14.25" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>13</v>
       </c>
@@ -13084,8 +13318,20 @@
       <c r="FD22" s="7">
         <v>40179.339999999997</v>
       </c>
+      <c r="FE22" s="7">
+        <v>41313.519999999997</v>
+      </c>
+      <c r="FF22" s="7">
+        <v>41686.019999999997</v>
+      </c>
+      <c r="FG22" s="7">
+        <v>43086.94</v>
+      </c>
+      <c r="FH22" s="7">
+        <v>44384.3</v>
+      </c>
     </row>
-    <row r="23" spans="1:160" ht="12.75" customHeight="1">
+    <row r="23" spans="1:164" ht="12.75" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>14</v>
       </c>
@@ -13566,8 +13812,20 @@
       <c r="FD23" s="7">
         <v>34149.089999999997</v>
       </c>
+      <c r="FE23" s="7">
+        <v>35322.370000000003</v>
+      </c>
+      <c r="FF23" s="7">
+        <v>36684.400000000001</v>
+      </c>
+      <c r="FG23" s="7">
+        <v>37754.57</v>
+      </c>
+      <c r="FH23" s="7">
+        <v>38009.64</v>
+      </c>
     </row>
-    <row r="24" spans="1:160" ht="12.75" customHeight="1">
+    <row r="24" spans="1:164" ht="12.75" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>15</v>
       </c>
@@ -14048,8 +14306,20 @@
       <c r="FD24" s="7">
         <v>104988.66</v>
       </c>
+      <c r="FE24" s="7">
+        <v>108632.3</v>
+      </c>
+      <c r="FF24" s="7">
+        <v>110504.73</v>
+      </c>
+      <c r="FG24" s="7">
+        <v>114012.82</v>
+      </c>
+      <c r="FH24" s="7">
+        <v>117778.6</v>
+      </c>
     </row>
-    <row r="25" spans="1:160" ht="12.75" customHeight="1">
+    <row r="25" spans="1:164" ht="12.75" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>16</v>
       </c>
@@ -14530,8 +14800,20 @@
       <c r="FD25" s="7">
         <v>98631.99</v>
       </c>
+      <c r="FE25" s="7">
+        <v>101836.79</v>
+      </c>
+      <c r="FF25" s="7">
+        <v>103798.49</v>
+      </c>
+      <c r="FG25" s="7">
+        <v>106052.54</v>
+      </c>
+      <c r="FH25" s="7">
+        <v>108226.57</v>
+      </c>
     </row>
-    <row r="26" spans="1:160" ht="12.75" customHeight="1">
+    <row r="26" spans="1:164" ht="12.75" customHeight="1">
       <c r="A26" s="3" t="s">
         <v>25</v>
       </c>
@@ -15012,8 +15294,20 @@
       <c r="FD26" s="10">
         <v>1618898.43</v>
       </c>
+      <c r="FE26" s="10">
+        <v>1647498.85</v>
+      </c>
+      <c r="FF26" s="10">
+        <v>1696991.68</v>
+      </c>
+      <c r="FG26" s="10">
+        <v>1729806.38</v>
+      </c>
+      <c r="FH26" s="10">
+        <v>1780370.93</v>
+      </c>
     </row>
-    <row r="27" spans="1:160" ht="12.75" customHeight="1">
+    <row r="27" spans="1:164" ht="12.75" customHeight="1">
       <c r="A27" s="4" t="s">
         <v>21</v>
       </c>
@@ -15494,8 +15788,20 @@
       <c r="FD27" s="7">
         <v>140558.46</v>
       </c>
+      <c r="FE27" s="7">
+        <v>142722.59</v>
+      </c>
+      <c r="FF27" s="7">
+        <v>143792.66</v>
+      </c>
+      <c r="FG27" s="7">
+        <v>143021.31</v>
+      </c>
+      <c r="FH27" s="7">
+        <v>142329.43</v>
+      </c>
     </row>
-    <row r="28" spans="1:160" ht="12.75" customHeight="1">
+    <row r="28" spans="1:164" ht="12.75" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>17</v>
       </c>
@@ -15976,8 +16282,20 @@
       <c r="FD28" s="7">
         <v>49124.86</v>
       </c>
+      <c r="FE28" s="7">
+        <v>50641.61</v>
+      </c>
+      <c r="FF28" s="7">
+        <v>52108.14</v>
+      </c>
+      <c r="FG28" s="7">
+        <v>54086.76</v>
+      </c>
+      <c r="FH28" s="7">
+        <v>55497.3</v>
+      </c>
     </row>
-    <row r="29" spans="1:160" ht="12.75" customHeight="1">
+    <row r="29" spans="1:164" ht="12.75" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>18</v>
       </c>
@@ -16458,8 +16776,20 @@
       <c r="FD29" s="7">
         <v>65706.899999999994</v>
       </c>
+      <c r="FE29" s="7">
+        <v>66749.06</v>
+      </c>
+      <c r="FF29" s="7">
+        <v>67143.149999999994</v>
+      </c>
+      <c r="FG29" s="7">
+        <v>67955.289999999994</v>
+      </c>
+      <c r="FH29" s="7">
+        <v>68981.350000000006</v>
+      </c>
     </row>
-    <row r="30" spans="1:160" ht="12.75" customHeight="1">
+    <row r="30" spans="1:164" ht="12.75" customHeight="1">
       <c r="A30" s="3" t="s">
         <v>19</v>
       </c>
@@ -16940,8 +17270,20 @@
       <c r="FD30" s="10">
         <v>1874288.65</v>
       </c>
+      <c r="FE30" s="10">
+        <v>1907612.11</v>
+      </c>
+      <c r="FF30" s="10">
+        <v>1960035.63</v>
+      </c>
+      <c r="FG30" s="10">
+        <v>1994869.74</v>
+      </c>
+      <c r="FH30" s="10">
+        <v>2047179.02</v>
+      </c>
     </row>
-    <row r="31" spans="1:160" ht="12.75" customHeight="1">
+    <row r="31" spans="1:164">
       <c r="A31" s="3" t="s">
         <v>28</v>
       </c>
@@ -17422,8 +17764,20 @@
       <c r="FD31" s="10">
         <v>29545.23</v>
       </c>
+      <c r="FE31" s="10">
+        <v>29841.54</v>
+      </c>
+      <c r="FF31" s="10">
+        <v>30843.8</v>
+      </c>
+      <c r="FG31" s="10">
+        <v>31392.35</v>
+      </c>
+      <c r="FH31" s="10">
+        <v>32307.43</v>
+      </c>
     </row>
-    <row r="32" spans="1:160" ht="12.75" customHeight="1">
+    <row r="32" spans="1:164">
       <c r="A32" s="3" t="s">
         <v>29</v>
       </c>
@@ -17904,29 +18258,41 @@
       <c r="FD32" s="10">
         <v>62476.29</v>
       </c>
+      <c r="FE32" s="10">
+        <v>63587.07</v>
+      </c>
+      <c r="FF32" s="10">
+        <v>65334.52</v>
+      </c>
+      <c r="FG32" s="10">
+        <v>66495.66</v>
+      </c>
+      <c r="FH32" s="10">
+        <v>68239.3</v>
+      </c>
     </row>
-    <row r="33" spans="1:16384" ht="17.25" customHeight="1">
-      <c r="A33" s="36" t="s">
+    <row r="33" spans="1:16384" ht="12.75" customHeight="1">
+      <c r="A33" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="B33" s="36"/>
-      <c r="C33" s="36"/>
-      <c r="D33" s="36"/>
-      <c r="E33" s="36"/>
-      <c r="F33" s="36"/>
-      <c r="G33" s="36"/>
-      <c r="H33" s="36"/>
-      <c r="I33" s="36"/>
+      <c r="B33" s="37"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="37"/>
+      <c r="H33" s="37"/>
+      <c r="I33" s="37"/>
     </row>
-    <row r="34" spans="1:16384" ht="15.75" customHeight="1">
+    <row r="34" spans="1:16384" ht="12.75" customHeight="1">
       <c r="A34" s="19" t="s">
         <v>27</v>
       </c>
       <c r="B34" s="20"/>
     </row>
-    <row r="35" spans="1:16384" ht="25.5" customHeight="1">
+    <row r="35" spans="1:16384" ht="26.25" customHeight="1">
       <c r="A35" s="35" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B35" s="35"/>
       <c r="C35" s="35"/>
@@ -17938,7 +18304,7 @@
     </row>
     <row r="36" spans="1:16384" ht="12.75" customHeight="1">
       <c r="A36" s="35" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B36" s="35"/>
       <c r="C36" s="35"/>
@@ -34325,7 +34691,8 @@
       <c r="XFD36" s="35"/>
     </row>
   </sheetData>
-  <mergeCells count="2050">
+  <mergeCells count="2051">
+    <mergeCell ref="A2:E2"/>
     <mergeCell ref="Q36:X36"/>
     <mergeCell ref="Y36:AF36"/>
     <mergeCell ref="AG36:AN36"/>
@@ -36397,10 +36764,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24.95" customHeight="1" thickBot="1">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="38"/>
+      <c r="B1" s="39"/>
     </row>
     <row r="2" spans="1:4" ht="24.95" customHeight="1" thickBot="1">
       <c r="A2" s="14" t="s">
@@ -36423,7 +36790,7 @@
         <v>36</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="24.95" customHeight="1">
@@ -36442,7 +36809,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="42.75" customHeight="1" thickBot="1">
+    <row r="7" spans="1:4" ht="42" customHeight="1" thickBot="1">
       <c r="A7" s="26" t="s">
         <v>41</v>
       </c>
@@ -36487,7 +36854,7 @@
       </c>
       <c r="D11" s="29"/>
     </row>
-    <row r="12" spans="1:4" ht="24.95" customHeight="1">
+    <row r="12" spans="1:4" ht="35.1" customHeight="1">
       <c r="A12" s="22" t="s">
         <v>51</v>
       </c>
@@ -36495,7 +36862,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="24.95" customHeight="1">
+    <row r="13" spans="1:4" ht="35.1" customHeight="1">
       <c r="A13" s="22" t="s">
         <v>53</v>
       </c>
@@ -36503,7 +36870,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="24.95" customHeight="1">
+    <row r="14" spans="1:4" ht="15.75" customHeight="1">
       <c r="A14" s="24" t="s">
         <v>55</v>
       </c>
@@ -36511,12 +36878,12 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="35.25" customHeight="1" thickBot="1">
+    <row r="15" spans="1:4" ht="50.1" customHeight="1" thickBot="1">
       <c r="A15" s="33" t="s">
         <v>56</v>
       </c>
       <c r="B15" s="34" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="24.95" customHeight="1"/>

</xml_diff>

<commit_message>
datos: actualización automática 2026-09-09
</commit_message>
<xml_diff>
--- a/idecba/canastas.xlsx
+++ b/idecba/canastas.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25635" windowHeight="3345"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25755" windowHeight="2955"/>
   </bookViews>
   <sheets>
     <sheet name="Canasta_cons_hogar1" sheetId="1" r:id="rId1"/>
@@ -314,7 +314,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>. Enero de 2013 / julio 2026</t>
+      <t>. Enero de 2013 / agosto 2026</t>
     </r>
   </si>
 </sst>
@@ -3399,7 +3399,7 @@
     <col min="79" max="16384" width="11.42578125" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:164" ht="15" customHeight="1">
+    <row r="1" spans="1:165" ht="15" customHeight="1">
       <c r="A1" s="15" t="s">
         <v>62</v>
       </c>
@@ -3426,7 +3426,7 @@
       <c r="V1" s="15"/>
       <c r="W1" s="15"/>
     </row>
-    <row r="2" spans="1:164" s="18" customFormat="1" ht="15" customHeight="1">
+    <row r="2" spans="1:165" s="18" customFormat="1" ht="15" customHeight="1">
       <c r="A2" s="36"/>
       <c r="B2" s="36"/>
       <c r="C2" s="36"/>
@@ -3451,7 +3451,7 @@
       <c r="V2" s="17"/>
       <c r="W2" s="17"/>
     </row>
-    <row r="3" spans="1:164" ht="15" customHeight="1">
+    <row r="3" spans="1:165" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>22</v>
       </c>
@@ -3944,8 +3944,11 @@
       <c r="FH3" s="5">
         <v>46204</v>
       </c>
+      <c r="FI3" s="5">
+        <v>46235</v>
+      </c>
     </row>
-    <row r="4" spans="1:164" ht="12.75" customHeight="1">
+    <row r="4" spans="1:165" ht="12.75" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
@@ -4438,8 +4441,11 @@
       <c r="FH4" s="7">
         <v>240504.8</v>
       </c>
+      <c r="FI4" s="7">
+        <v>247736.08</v>
+      </c>
     </row>
-    <row r="5" spans="1:164" ht="12.75" customHeight="1">
+    <row r="5" spans="1:165" ht="12.75" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
@@ -4932,8 +4938,11 @@
       <c r="FH5" s="7">
         <v>226072.85</v>
       </c>
+      <c r="FI5" s="7">
+        <v>230345.46</v>
+      </c>
     </row>
-    <row r="6" spans="1:164" ht="12.75" customHeight="1">
+    <row r="6" spans="1:165" ht="12.75" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
@@ -5426,8 +5435,11 @@
       <c r="FH6" s="7">
         <v>294091.18</v>
       </c>
+      <c r="FI6" s="7">
+        <v>295268.86</v>
+      </c>
     </row>
-    <row r="7" spans="1:164" ht="12.75" customHeight="1">
+    <row r="7" spans="1:165" ht="12.75" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>60</v>
       </c>
@@ -5920,8 +5932,11 @@
       <c r="FH7" s="7">
         <v>128513.31</v>
       </c>
+      <c r="FI7" s="7">
+        <v>131001.84</v>
+      </c>
     </row>
-    <row r="8" spans="1:164" ht="12.75" customHeight="1">
+    <row r="8" spans="1:165" ht="12.75" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>3</v>
       </c>
@@ -6414,8 +6429,11 @@
       <c r="FH8" s="7">
         <v>24892.34</v>
       </c>
+      <c r="FI8" s="7">
+        <v>25277.4</v>
+      </c>
     </row>
-    <row r="9" spans="1:164" ht="12.75" customHeight="1">
+    <row r="9" spans="1:165" ht="12.75" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
@@ -6908,8 +6926,11 @@
       <c r="FH9" s="8">
         <v>15030.22</v>
       </c>
+      <c r="FI9" s="8">
+        <v>15276.2</v>
+      </c>
     </row>
-    <row r="10" spans="1:164" ht="12.75" customHeight="1">
+    <row r="10" spans="1:165" ht="12.75" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>26</v>
       </c>
@@ -7402,8 +7423,11 @@
       <c r="FH10" s="8">
         <v>21328.84</v>
       </c>
+      <c r="FI10" s="8">
+        <v>21569.56</v>
+      </c>
     </row>
-    <row r="11" spans="1:164" ht="12.75" customHeight="1">
+    <row r="11" spans="1:165" ht="12.75" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
@@ -7896,8 +7920,11 @@
       <c r="FH11" s="8">
         <v>18789.5</v>
       </c>
+      <c r="FI11" s="8">
+        <v>19141.689999999999</v>
+      </c>
     </row>
-    <row r="12" spans="1:164" ht="12.75" customHeight="1">
+    <row r="12" spans="1:165" ht="12.75" customHeight="1">
       <c r="A12" s="3" t="s">
         <v>23</v>
       </c>
@@ -8390,8 +8417,11 @@
       <c r="FH12" s="10">
         <v>969223.04</v>
       </c>
+      <c r="FI12" s="10">
+        <v>985617.1</v>
+      </c>
     </row>
-    <row r="13" spans="1:164" ht="12.75" customHeight="1">
+    <row r="13" spans="1:165" ht="12.75" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>6</v>
       </c>
@@ -8884,8 +8914,11 @@
       <c r="FH13" s="7">
         <v>0</v>
       </c>
+      <c r="FI13" s="7">
+        <v>0</v>
+      </c>
     </row>
-    <row r="14" spans="1:164" ht="12.75" customHeight="1">
+    <row r="14" spans="1:165" ht="12.75" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>7</v>
       </c>
@@ -9378,8 +9411,11 @@
       <c r="FH14" s="7">
         <v>151417.81</v>
       </c>
+      <c r="FI14" s="7">
+        <v>156602.9</v>
+      </c>
     </row>
-    <row r="15" spans="1:164" ht="12.75" customHeight="1">
+    <row r="15" spans="1:165" ht="12.75" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>9</v>
       </c>
@@ -9872,8 +9908,11 @@
       <c r="FH15" s="7">
         <v>19435.02</v>
       </c>
+      <c r="FI15" s="7">
+        <v>20184.22</v>
+      </c>
     </row>
-    <row r="16" spans="1:164" ht="12.75" customHeight="1">
+    <row r="16" spans="1:165" ht="12.75" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>8</v>
       </c>
@@ -10366,8 +10405,11 @@
       <c r="FH16" s="7">
         <v>28413.98</v>
       </c>
+      <c r="FI16" s="7">
+        <v>28971.74</v>
+      </c>
     </row>
-    <row r="17" spans="1:164" ht="12.75" customHeight="1">
+    <row r="17" spans="1:165" ht="12.75" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>10</v>
       </c>
@@ -10860,8 +10902,11 @@
       <c r="FH17" s="7">
         <v>46838.53</v>
       </c>
+      <c r="FI17" s="7">
+        <v>48243.69</v>
+      </c>
     </row>
-    <row r="18" spans="1:164" ht="12.75" customHeight="1">
+    <row r="18" spans="1:165" ht="12.75" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -11354,8 +11399,11 @@
       <c r="FH18" s="7">
         <v>61810.09</v>
       </c>
+      <c r="FI18" s="7">
+        <v>63651.58</v>
+      </c>
     </row>
-    <row r="19" spans="1:164" ht="12.75" customHeight="1">
+    <row r="19" spans="1:165" ht="12.75" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>11</v>
       </c>
@@ -11848,8 +11896,11 @@
       <c r="FH19" s="7">
         <v>90970.64</v>
       </c>
+      <c r="FI19" s="7">
+        <v>92599.64</v>
+      </c>
     </row>
-    <row r="20" spans="1:164" ht="12.75" customHeight="1">
+    <row r="20" spans="1:165" ht="12.75" customHeight="1">
       <c r="A20" s="3" t="s">
         <v>24</v>
       </c>
@@ -12342,8 +12393,11 @@
       <c r="FH20" s="10">
         <v>1368109.1</v>
       </c>
+      <c r="FI20" s="10">
+        <v>1395870.87</v>
+      </c>
     </row>
-    <row r="21" spans="1:164" ht="12.75" customHeight="1">
+    <row r="21" spans="1:165" ht="12.75" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>12</v>
       </c>
@@ -12836,8 +12890,11 @@
       <c r="FH21" s="7">
         <v>103862.72</v>
       </c>
+      <c r="FI21" s="7">
+        <v>104033.45</v>
+      </c>
     </row>
-    <row r="22" spans="1:164" ht="14.25" customHeight="1">
+    <row r="22" spans="1:165" ht="14.25" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>13</v>
       </c>
@@ -13330,8 +13387,11 @@
       <c r="FH22" s="7">
         <v>44384.3</v>
       </c>
+      <c r="FI22" s="7">
+        <v>44648.26</v>
+      </c>
     </row>
-    <row r="23" spans="1:164" ht="12.75" customHeight="1">
+    <row r="23" spans="1:165" ht="12.75" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>14</v>
       </c>
@@ -13824,8 +13884,11 @@
       <c r="FH23" s="7">
         <v>38009.64</v>
       </c>
+      <c r="FI23" s="7">
+        <v>38819.599999999999</v>
+      </c>
     </row>
-    <row r="24" spans="1:164" ht="12.75" customHeight="1">
+    <row r="24" spans="1:165" ht="12.75" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>15</v>
       </c>
@@ -14318,8 +14381,11 @@
       <c r="FH24" s="7">
         <v>117778.6</v>
       </c>
+      <c r="FI24" s="7">
+        <v>121423.94</v>
+      </c>
     </row>
-    <row r="25" spans="1:164" ht="12.75" customHeight="1">
+    <row r="25" spans="1:165" ht="12.75" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>16</v>
       </c>
@@ -14812,8 +14878,11 @@
       <c r="FH25" s="7">
         <v>108226.57</v>
       </c>
+      <c r="FI25" s="7">
+        <v>110916.04</v>
+      </c>
     </row>
-    <row r="26" spans="1:164" ht="12.75" customHeight="1">
+    <row r="26" spans="1:165" ht="12.75" customHeight="1">
       <c r="A26" s="3" t="s">
         <v>25</v>
       </c>
@@ -15306,8 +15375,11 @@
       <c r="FH26" s="10">
         <v>1780370.93</v>
       </c>
+      <c r="FI26" s="10">
+        <v>1815712.16</v>
+      </c>
     </row>
-    <row r="27" spans="1:164" ht="12.75" customHeight="1">
+    <row r="27" spans="1:165" ht="12.75" customHeight="1">
       <c r="A27" s="4" t="s">
         <v>21</v>
       </c>
@@ -15800,8 +15872,11 @@
       <c r="FH27" s="7">
         <v>142329.43</v>
       </c>
+      <c r="FI27" s="7">
+        <v>140813.51999999999</v>
+      </c>
     </row>
-    <row r="28" spans="1:164" ht="12.75" customHeight="1">
+    <row r="28" spans="1:165" ht="12.75" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>17</v>
       </c>
@@ -16294,8 +16369,11 @@
       <c r="FH28" s="7">
         <v>55497.3</v>
       </c>
+      <c r="FI28" s="7">
+        <v>56218.94</v>
+      </c>
     </row>
-    <row r="29" spans="1:164" ht="12.75" customHeight="1">
+    <row r="29" spans="1:165" ht="12.75" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>18</v>
       </c>
@@ -16788,8 +16866,11 @@
       <c r="FH29" s="7">
         <v>68981.350000000006</v>
       </c>
+      <c r="FI29" s="7">
+        <v>70100.45</v>
+      </c>
     </row>
-    <row r="30" spans="1:164" ht="12.75" customHeight="1">
+    <row r="30" spans="1:165" ht="12.75" customHeight="1">
       <c r="A30" s="3" t="s">
         <v>19</v>
       </c>
@@ -17282,8 +17363,11 @@
       <c r="FH30" s="10">
         <v>2047179.02</v>
       </c>
+      <c r="FI30" s="10">
+        <v>2082845.07</v>
+      </c>
     </row>
-    <row r="31" spans="1:164">
+    <row r="31" spans="1:165" ht="15" customHeight="1">
       <c r="A31" s="3" t="s">
         <v>28</v>
       </c>
@@ -17776,8 +17860,11 @@
       <c r="FH31" s="10">
         <v>32307.43</v>
       </c>
+      <c r="FI31" s="10">
+        <v>32853.9</v>
+      </c>
     </row>
-    <row r="32" spans="1:164">
+    <row r="32" spans="1:165" ht="15" customHeight="1">
       <c r="A32" s="3" t="s">
         <v>29</v>
       </c>
@@ -18269,6 +18356,9 @@
       </c>
       <c r="FH32" s="10">
         <v>68239.3</v>
+      </c>
+      <c r="FI32" s="10">
+        <v>69428.17</v>
       </c>
     </row>
     <row r="33" spans="1:16384" ht="12.75" customHeight="1">
@@ -36809,7 +36899,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="42" customHeight="1" thickBot="1">
+    <row r="7" spans="1:4" ht="43.5" customHeight="1" thickBot="1">
       <c r="A7" s="26" t="s">
         <v>41</v>
       </c>
@@ -36870,7 +36960,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15.75" customHeight="1">
+    <row r="14" spans="1:4" ht="15" customHeight="1">
       <c r="A14" s="24" t="s">
         <v>55</v>
       </c>

</xml_diff>